<commit_message>
Swaptions (Bachelier, QuantLib reference) and FX vanna-volga smile from ATM/RR/BF
</commit_message>
<xml_diff>
--- a/outputs/2026-10-15/valuation_report.xlsx
+++ b/outputs/2026-10-15/valuation_report.xlsx
@@ -968,7 +968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -985,6 +985,7 @@
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1058,6 +1059,11 @@
           <t>vega_1pt</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>vega_1bp</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1108,6 +1114,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr"/>
       <c r="N2" s="4" t="inlineStr"/>
+      <c r="O2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1158,6 +1165,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr"/>
       <c r="N3" s="4" t="inlineStr"/>
+      <c r="O3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1208,6 +1216,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr"/>
       <c r="N4" s="4" t="inlineStr"/>
+      <c r="O4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1258,6 +1267,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr"/>
       <c r="N5" s="4" t="inlineStr"/>
+      <c r="O5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1308,6 +1318,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr"/>
       <c r="N6" s="4" t="inlineStr"/>
+      <c r="O6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1358,6 +1369,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr"/>
       <c r="N7" s="4" t="inlineStr"/>
+      <c r="O7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1408,6 +1420,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr"/>
       <c r="N8" s="4" t="inlineStr"/>
+      <c r="O8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1458,6 +1471,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr"/>
       <c r="N9" s="4" t="inlineStr"/>
+      <c r="O9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1508,6 +1522,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr"/>
       <c r="N10" s="4" t="inlineStr"/>
+      <c r="O10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1558,6 +1573,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr"/>
       <c r="N11" s="4" t="inlineStr"/>
+      <c r="O11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1610,6 +1626,7 @@
         <v>132005.259657203</v>
       </c>
       <c r="N12" s="4" t="inlineStr"/>
+      <c r="O12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1662,6 +1679,7 @@
         <v>-327713.5653652724</v>
       </c>
       <c r="N13" s="4" t="inlineStr"/>
+      <c r="O13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1714,6 +1732,7 @@
         <v>194553.2006508472</v>
       </c>
       <c r="N14" s="4" t="inlineStr"/>
+      <c r="O14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1766,6 +1785,7 @@
         <v>-101363.5470532727</v>
       </c>
       <c r="N15" s="4" t="inlineStr"/>
+      <c r="O15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1818,6 +1838,7 @@
         <v>157887.2864024627</v>
       </c>
       <c r="N16" s="4" t="inlineStr"/>
+      <c r="O16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1841,16 +1862,16 @@
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>119873.2775867174</v>
+        <v>119977.6623178743</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>120121.4491581641</v>
+        <v>120225.859055702</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-248.1715714466263</v>
+        <v>-248.1967378277041</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>-0.01567906532886108</v>
+        <v>-0.01567171393514353</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1858,20 +1879,21 @@
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>119873.2775867174</v>
+        <v>119977.6623178743</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>-56.71557522904186</v>
+        <v>-59.31778237826074</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>55.5828078402119</v>
+        <v>58.18534698987787</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>78158.58863030442</v>
+        <v>81776.10115407041</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>15828.21209308995</v>
-      </c>
+        <v>15837.24274542349</v>
+      </c>
+      <c r="O17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1895,16 +1917,16 @@
         </is>
       </c>
       <c r="E18" s="4" t="n">
-        <v>101813.0715448218</v>
+        <v>129899.4198868644</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>101754.322377721</v>
+        <v>129841.3194287837</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>58.74916710075922</v>
+        <v>58.10045808073482</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>0.001627017016432924</v>
+        <v>0.001690839978827537</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1912,20 +1934,21 @@
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>101813.0715448218</v>
+        <v>129899.4198868644</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>118.7069738969003</v>
+        <v>106.9906548367871</v>
       </c>
       <c r="L18" s="4" t="n">
-        <v>-121.2732455796067</v>
+        <v>-110.3191086637962</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>-39018.77530594695</v>
+        <v>-36274.47533187536</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>36108.51423641594</v>
-      </c>
+        <v>34361.89042621458</v>
+      </c>
+      <c r="O18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1949,16 +1972,16 @@
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>-158913.7926811358</v>
+        <v>-150927.0613590237</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>-159337.7013961996</v>
+        <v>-151339.5797442901</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>423.9087150637351</v>
+        <v>412.5183852663904</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>0.009456907598720232</v>
+        <v>0.00930295410556063</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1966,20 +1989,21 @@
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>-158913.7926811358</v>
+        <v>-150927.0613590237</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>241.8276256110694</v>
+        <v>234.7526863012463</v>
       </c>
       <c r="L19" s="4" t="n">
-        <v>-234.0012802354468</v>
+        <v>-227.3662585262791</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>-54182.50375527615</v>
+        <v>-53515.92232647844</v>
       </c>
       <c r="N19" s="4" t="n">
-        <v>-44825.29945847215</v>
-      </c>
+        <v>-44342.73033979785</v>
+      </c>
+      <c r="O19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2003,16 +2027,16 @@
         </is>
       </c>
       <c r="E20" s="4" t="n">
-        <v>-152738.9893474479</v>
+        <v>-158135.0336720072</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>-152613.3920023947</v>
+        <v>-158011.142626072</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>-125.5973450532474</v>
+        <v>-123.89104593519</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>-0.005145202000792561</v>
+        <v>-0.00515846425862998</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -2020,20 +2044,21 @@
         </is>
       </c>
       <c r="J20" s="4" t="n">
-        <v>-152738.9893474479</v>
+        <v>-158135.0336720072</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>-248.4857187101734</v>
+        <v>-221.5824099538149</v>
       </c>
       <c r="L20" s="4" t="n">
-        <v>263.632684389042</v>
+        <v>237.259154968051</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>23391.21470827315</v>
+        <v>20645.86146025689</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>-24410.57611224992</v>
-      </c>
+        <v>-24017.040677935</v>
+      </c>
+      <c r="O20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2057,16 +2082,16 @@
         </is>
       </c>
       <c r="E21" s="4" t="n">
-        <v>497581.3661568928</v>
+        <v>492407.2611426145</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>498095.9041374864</v>
+        <v>492917.9630980644</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>-514.5379805935663</v>
+        <v>-510.701955449942</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>-0.007141290470356128</v>
+        <v>-0.006998074243598721</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -2074,19 +2099,232 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>497581.3661568928</v>
+        <v>492407.2611426145</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>-1008.31345262687</v>
+        <v>-1062.618610213336</v>
       </c>
       <c r="L21" s="4" t="n">
-        <v>934.3405594197684</v>
+        <v>989.638052617549</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>70030.47864096501</v>
+        <v>74106.1937559045</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>72051.12055439287</v>
+        <v>72977.49890508683</v>
+      </c>
+      <c r="O21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>NBM-SWO-001</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SWPTN</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Bank A</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>551987.2558995166</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>551987.2558993883</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>1.282896846532822e-07</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>2.590124082387129e-11</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>731198.813866184</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>6880.180702718673</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="4" t="inlineStr"/>
+      <c r="N22" s="4" t="inlineStr"/>
+      <c r="O22" s="4" t="n">
+        <v>4953.03238658153</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>NBM-SWO-002</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SWPTN</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Bank C</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>-44139.16974099607</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>-44139.16974099571</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>-3.637978807091713e-10</v>
+      </c>
+      <c r="H23" s="6" t="n">
+        <v>-4.153117487237627e-13</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>-58469.66250526935</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>1085.833288045302</v>
+      </c>
+      <c r="L23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="4" t="inlineStr"/>
+      <c r="N23" s="4" t="inlineStr"/>
+      <c r="O23" s="4" t="n">
+        <v>-875.9633740849094</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>NBM-SWO-003</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SWPTN</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Bank E</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>1246935.671853965</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>1246935.671854194</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>-2.298038452863693e-07</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>-1.486943668694637e-11</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>1246935.671853965</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>-12635.3170910764</v>
+      </c>
+      <c r="M24" s="4" t="inlineStr"/>
+      <c r="N24" s="4" t="inlineStr"/>
+      <c r="O24" s="4" t="n">
+        <v>15454.77815498621</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>NBM-SWO-004</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SWPTN</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Bank D</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>-134735.9021411029</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>-134735.902141131</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>2.811430022120476e-08</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>1.415271968819973e-11</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>-134735.9021411029</v>
+      </c>
+      <c r="K25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="4" t="n">
+        <v>-3746.402908673132</v>
+      </c>
+      <c r="M25" s="4" t="inlineStr"/>
+      <c r="N25" s="4" t="inlineStr"/>
+      <c r="O25" s="4" t="n">
+        <v>-1986.494528302283</v>
       </c>
     </row>
   </sheetData>
@@ -2100,7 +2338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2978,16 +3216,16 @@
         </is>
       </c>
       <c r="E17" s="4" t="n">
-        <v>119873.2775867174</v>
+        <v>119977.6623178743</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>120381.7247403665</v>
+        <v>120486.3995617399</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>508.447153649031</v>
+        <v>508.7372438656312</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>3957.053023272489</v>
+        <v>3959.310686355871</v>
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
@@ -2997,7 +3235,7 @@
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" s="4" t="n">
-        <v>508.447153649031</v>
+        <v>508.7372438656312</v>
       </c>
       <c r="M17" t="inlineStr"/>
     </row>
@@ -3023,16 +3261,16 @@
         </is>
       </c>
       <c r="E18" s="4" t="n">
-        <v>101813.0715448218</v>
+        <v>129899.4198868644</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>157039.6844933707</v>
+        <v>182480.0407319393</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>55226.61294854889</v>
+        <v>52580.62084507488</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>9027.128559103985</v>
+        <v>8590.472606553645</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -3050,7 +3288,7 @@
         </is>
       </c>
       <c r="L18" s="4" t="n">
-        <v>-1145.758404795779</v>
+        <v>-1120.520194034441</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -3080,16 +3318,16 @@
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>-158913.7926811358</v>
+        <v>-150927.0613590237</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>-176843.9124645247</v>
+        <v>-168664.1534949428</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>-17930.11978338886</v>
+        <v>-17737.09213591914</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>11206.32486461804</v>
+        <v>11085.68258494946</v>
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
@@ -3137,16 +3375,16 @@
         </is>
       </c>
       <c r="E20" s="4" t="n">
-        <v>-152738.9893474479</v>
+        <v>-158135.0336720072</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>-152013.8257573305</v>
+        <v>-157421.5608165564</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>725.163590117445</v>
+        <v>713.4728554508765</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>6102.644028062481</v>
+        <v>6004.26016948375</v>
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
@@ -3156,7 +3394,7 @@
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
       <c r="L20" s="4" t="n">
-        <v>725.163590117445</v>
+        <v>713.4728554508765</v>
       </c>
       <c r="M20" t="inlineStr"/>
     </row>
@@ -3182,16 +3420,16 @@
         </is>
       </c>
       <c r="E21" s="4" t="n">
-        <v>497581.3661568928</v>
+        <v>492407.2611426145</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>621976.7076961159</v>
+        <v>615509.0764282681</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>124395.3415392232</v>
+        <v>123101.8152856536</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>18012.78013859822</v>
+        <v>18244.37472627171</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
@@ -3214,6 +3452,222 @@
       <c r="M21" t="inlineStr">
         <is>
           <t>Booking break: confirm notional against the confirmation; escalate to operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>NBM-SWO-001</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Bank A</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>SWPTN</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>551987.2558995166</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>551971.3739778124</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>-15.88192170427646</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>4953.03238658153</v>
+      </c>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t>WITHIN_TOLERANCE</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" s="4" t="n">
+        <v>-15.88192170427646</v>
+      </c>
+      <c r="M22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>NBM-SWO-002</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Bank C</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>SWPTN</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>-44139.16974099607</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>-49436.6639897958</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>-5297.494248799732</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>VOL</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>dealer normal vol about +6.0bp from ours</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="n">
+        <v>42.42786858393811</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Request the dealer's vol for this expiry/strike and compare with our surface</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>NBM-SWO-003</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Bank E</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>SWPTN</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>1246935.671853965</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>1126950.463903606</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>-119985.207950359</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>15454.77815498621</v>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>EXPLAINED</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>PRIOR_DAY</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>matches a mark off 2026-10-14 curves and spot</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Ask the dealer for the curve/spot snapshot date; re-request today's mark</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>NBM-SWO-004</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Bank D</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>SWPTN</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>-134735.9021411029</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>-137715.6439335563</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>-2979.741792453424</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>1986.494528302283</v>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>BID_SIDE</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>gap = 1.5bp normal vol against us (bid/offer side)</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Ask whether the mark is mid or bid/offer; request a mid mark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SONIA-SOFR cross-currency basis swap with notional exchanges; QuantLib leg reference
</commit_message>
<xml_diff>
--- a/outputs/2026-10-15/valuation_report.xlsx
+++ b/outputs/2026-10-15/valuation_report.xlsx
@@ -968,7 +968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O25"/>
+  <dimension ref="A1:O27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2327,6 +2327,112 @@
         <v>-1986.494528302283</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>NBM-XCY-001</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>XCCY</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Bank B</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>-110587.8031512722</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>-110587.8031512722</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>-110587.8031512722</v>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>-3.725290298461914e-09</v>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="4" t="n">
+        <v>266481.2204540558</v>
+      </c>
+      <c r="N26" s="4" t="inlineStr"/>
+      <c r="O26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>NBM-XCY-002</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>XCCY</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Bank E</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>431387.6903665252</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>431387.6903665215</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>3.725290298461914e-09</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>1.869603424995306e-12</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>431387.6903665252</v>
+      </c>
+      <c r="K27" s="4" t="n">
+        <v>-25.11622706800699</v>
+      </c>
+      <c r="L27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="4" t="n">
+        <v>-199255.6415257566</v>
+      </c>
+      <c r="N27" s="4" t="inlineStr"/>
+      <c r="O27" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2338,7 +2444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:M27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3671,6 +3777,108 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>NBM-XCY-001</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Bank B</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>XCCY</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>-110587.8031512722</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>110587.8031512722</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>221175.6063025445</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>5329.624409081116</v>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>EXPLAINED</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>DIRECTION</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>matches the opposite direction</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Booking break: confirm direction against the confirmation; escalate to operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>NBM-XCY-002</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Bank E</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>XCCY</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>431387.6903665252</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>431348.4434663713</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>-39.24690015387023</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>3985.112830515131</v>
+      </c>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>WITHIN_TOLERANCE</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" s="4" t="n">
+        <v>-39.24690015387023</v>
+      </c>
+      <c r="M27" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>